<commit_message>
actualizacion fuentes de proyectos en evaluación
</commit_message>
<xml_diff>
--- a/downloads/base_completa.xlsx
+++ b/downloads/base_completa.xlsx
@@ -2024,7 +2024,7 @@
       </c>
       <c r="V15" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gobier [https://www.salta.gob.ar/prensa/noticias/vinculos-con-empresa-minera-china-para-el-ingreso-de-productos-saltenios-al-pais-asiatico-104841]; o de Salta [https://www.casarosada.gob.ar/slider-principal/50224-el-presidente-se-reunio-con-autoridades-de-una-empresa-china-que-desarrolla-proyectos-de-extraccion-de-litio-en-salta]; Casa Rosada [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; I; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gobierno de Salta [https://www.salta.gob.ar/prensa/noticias/vinculos-con-empresa-minera-china-para-el-ingreso-de-productos-saltenios-al-pais-asiatico-104841]; Casa Rosada [https://www.casarosada.gob.ar/slider-principal/50224-el-presidente-se-reunio-con-autoridades-de-una-empresa-china-que-desarrolla-proyectos-de-extraccion-de-litio-en-salta]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W15" t="inlineStr">
@@ -2097,7 +2097,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; I [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; fobae [https://rionegro.gov.ar/articulo/53275/rio-negro-fortalece-su-rol-en-el-abastecimiento-de-arena-para-vaca-muerta]; Gobier; o de Río Negro; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; Gobierno de Río Negro [https://rionegro.gov.ar/articulo/53275/rio-negro-fortalece-su-rol-en-el-abastecimiento-de-arena-para-vaca-muerta]</t>
         </is>
       </c>
       <c r="W16" t="inlineStr">
@@ -2170,7 +2170,7 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gobier [https://www.neuqueninforma.gob.ar/noticias/2026/04/23/256641-neuquen-suma-un-nuevo-megaproyecto-al-rigi-con-apoyo-de-gyp]; o de Neuqué [https://econojournal.com.ar/oilgas/pluspetrol-solicito-la-adhesion-al-rigi-para-el-bloque-bajo-del-choique-la-invernada-con-una-inversion-de-us12-000-millones/]; Eco [https://x.com/LuisCaputoAR/status/2047621135127269495]; oJour [https://www.clarin.com/economia/rigi-vaca-muerta-pluspetrol-presento-inversiones-us-12000-millones-campo-compro-exxon_0_gYALiNgXD0.html]; al; Luis Caputo; Clarí; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gobierno de Neuquén [https://www.neuqueninforma.gob.ar/noticias/2026/04/23/256641-neuquen-suma-un-nuevo-megaproyecto-al-rigi-con-apoyo-de-gyp]; EconoJournal [https://econojournal.com.ar/oilgas/pluspetrol-solicito-la-adhesion-al-rigi-para-el-bloque-bajo-del-choique-la-invernada-con-una-inversion-de-us12-000-millones/]; Luis Caputo [https://x.com/LuisCaputoAR/status/2047621135127269495]; Clarín [https://www.clarin.com/economia/rigi-vaca-muerta-pluspetrol-presento-inversiones-us-12000-millones-campo-compro-exxon_0_gYALiNgXD0.html]</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
@@ -2356,7 +2356,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Oldelval [https://www.oldelval.com/oldelval-inicia-la-etapa-constructiva-del-proyecto-duplicar-norte/]; I [https://www.oldelval.com/oldelval-confirmo-la-ejecucion-del-proyecto-duplicar-norte/]; fobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Oldelval [https://www.oldelval.com/oldelval-inicia-la-etapa-constructiva-del-proyecto-duplicar-norte/]; Oldelval [https://www.oldelval.com/oldelval-confirmo-la-ejecucion-del-proyecto-duplicar-norte/]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W19" t="inlineStr">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gle [https://www.glencore.com/media-and-insights/news/glencore-submits-RIGI-applications-in-respect-of-its-argentine-copper-projects]; core [https://x.com/LuisCaputoAR/status/1957458679835594969]; Luis Caputo [https://www.reuters.com/latam/negocio/7X5ZW2SXG5IYNBUILMTT6GMS6U-2025-08-21/]; Reuters [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; I; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Glencore [https://www.glencore.com/media-and-insights/news/glencore-submits-RIGI-applications-in-respect-of-its-argentine-copper-projects]; Luis Caputo [https://x.com/LuisCaputoAR/status/1957458679835594969]; Reuters [https://www.reuters.com/latam/negocio/7X5ZW2SXG5IYNBUILMTT6GMS6U-2025-08-21/]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W20" t="inlineStr">
@@ -2502,7 +2502,7 @@
       </c>
       <c r="V21" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Chevro [https://www.chevron.com/worldwide/argentina]; I [https://www.infobae.com/economia/2026/06/02/chevron-presento-un-megaproyecto-bajo-el-rigi-para-invertir-usd-13800-millones-en-vaca-muerta/]; fobae [https://www.clarin.com/economia/megainversion-vaca-muerta-chevron-presento-pedido-rigi-us-13800-millones_0_EXuEOYbjiy.html]; Clarí; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Chevron [https://www.chevron.com/worldwide/argentina]; Infobae [https://www.infobae.com/economia/2026/06/02/chevron-presento-un-megaproyecto-bajo-el-rigi-para-invertir-usd-13800-millones-en-vaca-muerta/]; Clarín [https://www.clarin.com/economia/megainversion-vaca-muerta-chevron-presento-pedido-rigi-us-13800-millones_0_EXuEOYbjiy.html]</t>
         </is>
       </c>
       <c r="W21" t="inlineStr">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Mi [https://www.argentina.gob.ar/normativa/nacional/resoluci%C3%B3n-39-2025-415411/texto]; isterio de Eco [https://www.nca.com.ar/Nuestra-red]; omía / Boletí [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; Oficial; Nuevo Ce; tral Arge; ti; o; I; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Ministerio de Economía / Boletín Oficial [https://www.argentina.gob.ar/normativa/nacional/resoluci%C3%B3n-39-2025-415411/texto]; Nuevo Central Argentino [https://www.nca.com.ar/Nuestra-red]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
@@ -2645,7 +2645,7 @@
       </c>
       <c r="V23" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Te [https://www.tenaris.com/en/news/2025/tenaris-begins-construction-of-second-wind-farm-in-argentina]; aris [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; I; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Tenaris [https://www.tenaris.com/en/news/2025/tenaris-begins-construction-of-second-wind-farm-in-argentina]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W23" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="V24" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Techi [https://www.techint.com/es/nuestros-proyectos/los-toldos-ii-este]; t I [https://vacamuertanews.com/amp/a-30-km-de-rincon-de-los-sauces-tecpetrol-y-gyp-lanzan-un-megaproyecto-de-shale-oil-con-380-pozos.htm]; ge [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; iería y Co; strucció; Vaca Muerta News; I; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Techint Ingeniería y Construcción [https://www.techint.com/es/nuestros-proyectos/los-toldos-ii-este]; Vaca Muerta News [https://vacamuertanews.com/amp/a-30-km-de-rincon-de-los-sauces-tecpetrol-y-gyp-lanzan-un-megaproyecto-de-shale-oil-con-380-pozos.htm]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W24" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="V25" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gobier [https://www.salta.gob.ar/prensa/noticias/avanza-en-salta-el-proyecto-de-litio-pozuelos-pastos-grandes-104827]; o de Salta [https://investors.lithium-argentina.com/news-releases/news-release-details/lithium-argentina-reports-fourth-quarter-and-full-year-2025]; Lithium Arge [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; ti; a; I; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gobierno de Salta [https://www.salta.gob.ar/prensa/noticias/avanza-en-salta-el-proyecto-de-litio-pozuelos-pastos-grandes-104827]; Lithium Argentina [https://investors.lithium-argentina.com/news-releases/news-release-details/lithium-argentina-reports-fourth-quarter-and-full-year-2025]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W25" t="inlineStr">
@@ -3090,7 +3090,7 @@
       </c>
       <c r="V28" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Rio Ti [https://www.riotinto.com/en/news/releases/2025/rio-tinto-confirmed-as-preferred-partner-on-world-class-salares-altoandinos-lithium-project]; to [https://www.infobae.com/economia/2025/10/07/hay-mas-de-usd-18000-millones-a-la-espera-de-aprobacion-en-proyectos-del-rigi/]; I [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Rio Tinto [https://www.riotinto.com/en/news/releases/2025/rio-tinto-confirmed-as-preferred-partner-on-world-class-salares-altoandinos-lithium-project]; Infobae [https://www.infobae.com/economia/2025/10/07/hay-mas-de-usd-18000-millones-a-la-espera-de-aprobacion-en-proyectos-del-rigi/]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W28" t="inlineStr">
@@ -3384,7 +3384,7 @@
       </c>
       <c r="V31" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; GeoPark [https://www.geo-park.com/es/news/geopark-solicita-adhesion-al-rigi-por-proyecto-de-inversion/]; Eco [https://econojournal.com.ar/oilgas/geopark-presenta-al-rigi-una-inversion-por-us1-000-millones-para-un-hub-petrolero-en-vaca-muerta/]; oJour; al; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; GeoPark [https://www.geo-park.com/es/news/geopark-solicita-adhesion-al-rigi-por-proyecto-de-inversion/]; EconoJournal [https://econojournal.com.ar/oilgas/geopark-presenta-al-rigi-una-inversion-por-us1-000-millones-para-un-hub-petrolero-en-vaca-muerta/]</t>
         </is>
       </c>
       <c r="W31" t="inlineStr">
@@ -3633,7 +3633,7 @@
       </c>
       <c r="V34" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Eco [https://econojournal.com.ar/oilgas/vaca-muerta-mega-se-presenta-al-rigi-con-una-inversion-de-us360-millones-en-su-planta-de-separacion-de-liquidos-del-gas/]; oJour [https://www.ingenierowhite.com/2026/07/31/mega-obtuvo-la-aprobacion-de-su-proyecto-de-inversion-bajo-el-rigi/]; al [https://x.com/LuisCaputoAR/status/2083255389399744911]; Compañía MEGA; Luis Caputo; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; EconoJournal [https://econojournal.com.ar/oilgas/vaca-muerta-mega-se-presenta-al-rigi-con-una-inversion-de-us360-millones-en-su-planta-de-separacion-de-liquidos-del-gas/]; Compañía MEGA [https://www.ingenierowhite.com/2026/07/31/mega-obtuvo-la-aprobacion-de-su-proyecto-de-inversion-bajo-el-rigi/]; Luis Caputo [https://x.com/LuisCaputoAR/status/2083255389399744911]</t>
         </is>
       </c>
       <c r="W34" t="inlineStr">
@@ -3706,7 +3706,7 @@
       </c>
       <c r="V35" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gle [https://www.glencore.com/media-and-insights/news/glencore-submits-RIGI-applications-in-respect-of-its-argentine-copper-projects]; core [https://x.com/LuisCaputoAR/status/1957458679835594969]; Luis Caputo [https://www.reuters.com/latam/negocio/7X5ZW2SXG5IYNBUILMTT6GMS6U-2025-08-21/]; Reuters [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; I; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Glencore [https://www.glencore.com/media-and-insights/news/glencore-submits-RIGI-applications-in-respect-of-its-argentine-copper-projects]; Luis Caputo [https://x.com/LuisCaputoAR/status/1957458679835594969]; Reuters [https://www.reuters.com/latam/negocio/7X5ZW2SXG5IYNBUILMTT6GMS6U-2025-08-21/]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W35" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="V36" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Pampa E [https://ri.pampa.com/en/press-release/pampa-energia-announces-its-entry-into-the-fertilizer-business-with-the-construction-of-latin-americas-largest-urea-plant/]; ergía [https://disclosures.ifc.org/project-detail/ED/52106/fer-il-p]; I [https://www.cronista.com/negocios/fertil-pampa-se-presenta-al-rigi-con-una-inversion-de-us-2400-millones-para-producir-fertilizantes/]; ter [https://www.lanacion.com.ar/economia/campo/invertiria-us2400-millones-una-empresa-de-marcelo-mindlin-pidio-ingresar-al-rigi-para-producir-nid23042026/]; atio; al Fi; a; ce Corporatio; El Cro; ista; La Nació; Luis Caputo; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Pampa Energía [https://ri.pampa.com/en/press-release/pampa-energia-announces-its-entry-into-the-fertilizer-business-with-the-construction-of-latin-americas-largest-urea-plant/]; International Finance Corporation [https://disclosures.ifc.org/project-detail/ED/52106/fer-il-p]; El Cronista [https://www.cronista.com/negocios/fertil-pampa-se-presenta-al-rigi-con-una-inversion-de-us-2400-millones-para-producir-fertilizantes/]; La Nación [https://www.lanacion.com.ar/economia/campo/invertiria-us2400-millones-una-empresa-de-marcelo-mindlin-pidio-ingresar-al-rigi-para-producir-nid23042026/]; Luis Caputo</t>
         </is>
       </c>
       <c r="W36" t="inlineStr">
@@ -4078,7 +4078,7 @@
       </c>
       <c r="V39" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gobier [https://prensa.jujuy.gob.ar/jujuy/jujuy-se-afianza-como-productor-minerales-criticos-el-desarrollo-la-transicion-energetica-n120116]; o de Jujuy [https://eltribunodejujuy.com/informacion-general/2026-4-1-0-0-0-proyecto-de-litio-en-jujuy-busca-la-adhesion-al-rigi]; El Tribu [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]; o de Jujuy; I; fobae; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Gobierno de Jujuy [https://prensa.jujuy.gob.ar/jujuy/jujuy-se-afianza-como-productor-minerales-criticos-el-desarrollo-la-transicion-energetica-n120116]; El Tribuno de Jujuy [https://eltribunodejujuy.com/informacion-general/2026-4-1-0-0-0-proyecto-de-litio-en-jujuy-busca-la-adhesion-al-rigi]; Infobae [https://www.infobae.com/economia/2026/05/13/el-gobierno-aprobo-el-ingreso-al-rigi-de-la-ampliacion-del-gasoducto-perito-moreno-con-una-inversion-de-usd-550-millones/]</t>
         </is>
       </c>
       <c r="W39" t="inlineStr">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; YPF [https://www.instagram.com/p/DYX1JXjj-bC/]; Eco [https://econojournal.com.ar/destacada/ypf-presento-rigi-acelerar-produccion-petroleo-vaca-muerta/]; oJour [https://www.reuters.com/business/energy/argentinas-ypf-registers-25-bln-oil-project-rigi-investment-scheme-2026-05-15/]; al; Reuters; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; YPF [https://www.instagram.com/p/DYX1JXjj-bC/]; EconoJournal [https://econojournal.com.ar/destacada/ypf-presento-rigi-acelerar-produccion-petroleo-vaca-muerta/]; Reuters [https://www.reuters.com/business/energy/argentinas-ypf-registers-25-bln-oil-project-rigi-investment-scheme-2026-05-15/]</t>
         </is>
       </c>
       <c r="W40" t="inlineStr">
@@ -4224,7 +4224,7 @@
       </c>
       <c r="V41" t="inlineStr">
         <is>
-          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; Eco [https://econojournal.com.ar/oilgas/vista-energy-pidio-la-adhesion-al-rigi-para-un-proyecto-de-us-5-800-millones-en-vaca-muerta/]; oJour [https://www.sec.gov/Archives/edgar/data/1762506/000119312526306139/d151775dex1.htm]; al [https://www.ogj.com/exploration-development/news/55394130/vista-seeks-rigi-approval-for-58-billion-bandurria-norte-development]; Vista E; ergy / SEC; Oil &amp; Gas Jour; al; auditoría 2026-08-08</t>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; EconoJournal [https://econojournal.com.ar/oilgas/vista-energy-pidio-la-adhesion-al-rigi-para-un-proyecto-de-us-5-800-millones-en-vaca-muerta/]; Vista Energy / SEC [https://www.sec.gov/Archives/edgar/data/1762506/000119312526306139/d151775dex1.htm]; Oil &amp; Gas Journal [https://www.ogj.com/exploration-development/news/55394130/vista-seeks-rigi-approval-for-58-billion-bandurria-norte-development]</t>
         </is>
       </c>
       <c r="W41" t="inlineStr">

</xml_diff>

<commit_message>
Mejorar hitos, autoría y descargas
</commit_message>
<xml_diff>
--- a/downloads/base_completa.xlsx
+++ b/downloads/base_completa.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z41"/>
+  <dimension ref="A1:X41"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="16" max="16" width="20.7109375" style="2" customWidth="1"/>
@@ -485,16 +485,6 @@
           <t>Links fuentes (original)</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Clasificación preexistencia BO</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>Justificación preexistencia BO</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -598,16 +588,6 @@
           <t>Res. 676/2026, Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>La resolución describe la “Ampliación del Tramo I” del Gasoducto Perito Francisco Moreno, instalando compresoras para aumentar la capacidad de un gasoducto ya existente, lo cual prueba que el proyecto es una ampliación de un activo preexistente.</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -711,16 +691,6 @@
           <t>Res. 562/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>La resolución para el proyecto Diablillos detalla la construcción de una planta de procesamiento y obras asociadas para un yacimiento de oro y plata sin mencionar expansiones ni proyectos previos.</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -824,16 +794,6 @@
           <t>Res. 6/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>La norma del proyecto Carbonatos Profundos describe la exploración de las concesiones Gualcamayo 1 y 2 y la construcción de una planta de tratamiento, sin referencias a fases previas o ampliaciones.</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -937,16 +897,6 @@
           <t>Res. 1254/2025; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>La resolución del Parque Eólico Olavarría describe la instalación de un nuevo parque eólico de 180 MW y obras de conexión eléctrica. Aunque se mencionan ampliaciones de la red de transporte, estas se refieren al sistema eléctrico y no evidencian un parque eólico preexistente.</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1050,16 +1000,6 @@
           <t>Res. 1/2025, Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z6" t="inlineStr">
-        <is>
-          <t>La resolución del Parque Solar El Quemado y Anexos indica la construcción de un parque solar fotovoltaico de 305 MW desarrollado en dos etapas; no hay menciones a instalaciones solares previas ni a ampliaciones de un proyecto existente.</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1163,16 +1103,6 @@
           <t>Res. 559/2025; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>La resolución para la planta de Licuefacción de Gas Natural (FLNG) describe la instalación de una planta flotante de GNL y conexión a gasoductos, sin señalar etapas previas ni ampliaciones.</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1276,16 +1206,6 @@
           <t>Res. 1028/2025; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z8" t="inlineStr">
-        <is>
-          <t>El Proyecto Siderúrgico Argentino Sidersa consiste en construir y poner en marcha una nueva planta de acería y laminación de aceros largos; la resolución no indica ampliaciones de plantas existentes.</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1389,16 +1309,6 @@
           <t>Res. 801/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>La norma del proyecto PSJ Cobre Mendocino expone la construcción y operación de una nueva mina a cielo abierto y planta concentradora en el yacimiento San Jorge, sin referencias a fases anteriores ni instalaciones preexistentes.</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1502,16 +1412,6 @@
           <t>Res. 735/2025; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z10" t="inlineStr">
-        <is>
-          <t>La resolución del Proyecto Rincón detalla que la producción provendrá tanto de la planta Rincón 3000, con capacidad de 3.000 t de LCE, como de la construcción y operación de dos plantas “Rincón Full Potential” de 25.000 t cada una, mostrando que el proyecto amplía una planta existente.</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1615,16 +1515,6 @@
           <t>Res. 431/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y11" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z11" t="inlineStr">
-        <is>
-          <t>La resolución del proyecto “Expansión Fase 1B” señala que consiste en la ampliación del proyecto preexistente Fénix para incrementar la capacidad productiva de carbonato de litio en 9.500 t/año.</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1728,16 +1618,6 @@
           <t>Res. 1842/2025; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y12" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>La resolución del Proyecto Terminal Multipropósito Timbúes aprueba la construcción y operación de una nueva terminal portuaria compuesta por tres unidades logístico‑portuarias; la norma no menciona ninguna infraestructura portuaria previa.</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1841,16 +1721,6 @@
           <t>Res. 302/2025; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y13" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z13" t="inlineStr">
-        <is>
-          <t>La resolución del oleoducto VMOS describe la construcción de un oleoducto de 437 km y terminales de exportación para incrementar la capacidad de transporte de petróleo; no se mencionan ampliaciones de un oleoducto existente.</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1954,16 +1824,6 @@
           <t>Res. 413/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y14" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z14" t="inlineStr">
-        <is>
-          <t>La resolución para las Fases 8 y 9 del Sistema de Lixiviación en Valle de Mina Veladero señala que se trata de una ampliación de un proyecto preexistente (Fases 1–7), agregando nuevas fases al sistema de lixiviación.</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2286,16 +2146,6 @@
           <t>Res. 825/2026, Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y18" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t>La resolución del proyecto “Ampliación Cauchari Olaroz” indica que se trata de la ampliación de un proyecto preexistente de 40.000 t/año de LCE; se construirá infraestructura adicional para incrementar la capacidad en 45.000 t/año.</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2907,16 +2757,6 @@
           <t>Res. 1025/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y26" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z26" t="inlineStr">
-        <is>
-          <t>Se identifican signos fuertes de preexistencia. El Proyecto Rincón de Aranda no surge con la resolución publicada el 21/07/2026. Antes de esa fecha existían antecedentes societarios, operativos, financieros y ambientales: Pampa Energía adquirió el control total del bloque en 2023; la etapa inicial del plan aprobado se declara iniciada el 08/07/2024; en 2024 ya existían EIAs y audiencias públicas para la CPF, oleoductos y gasoductos asociados; en 2025 la empresa ya informaba inversiones, solicitud RIGI, producción y pozos en operación. Por lo tanto, corresponde clasificarlo como proyecto preexistente al anuncio/aprobación oficial, aunque formalizado y ampliado bajo el RIGI como PEELP.</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3020,16 +2860,6 @@
           <t>Res. 1157/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y27" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z27" t="inlineStr">
-        <is>
-          <t>Signos fuertes de preexistencia del Proyecto Sal de Oro II. POSCO Holdings aprobó la inversión de la segunda fase en octubre de 2022; en junio de 2023, antes del primer anuncio del RIGI, el Gobierno nacional y la empresa comunicaron el inicio de construcción de una planta de carbonato de litio de 23.000 toneladas anuales; y en abril de 2024 POSCO obtuvo financiamiento por hasta USD 668 millones para esa misma fase. Las coincidencias de empresa, localización, producto, capacidad y etapa indican que se trata sustancialmente del mismo proyecto incorporado posteriormente al régimen.</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3201,16 +3031,6 @@
           <t>Res. 1153/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y29" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z29" t="inlineStr">
-        <is>
-          <t>Se identifican signos muy fuertes de preexistencia. El proyecto aprobado bajo RIGI corresponde a LIEX S.A. Sucursal Dedicada en el Salar Tres Quebradas —3Q—, Catamarca. Aunque la Resolución 1153/2026 aprueba una inversión en activos computables por USD 594,136 millones para una planta de 40.000 t/año de carbonato de litio, el proyecto 3Q existía públicamente desde años previos: tuvo evaluación económica preliminar en 2017, estudio de factibilidad en 2021, acuerdo provincial ratificado por ley en 2022, adquisición por Zijin/LIEX en 2022, infraestructura eléctrica asociada tramitada desde 2023–2024 y primera fase en producción desde septiembre de 2025.</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3314,16 +3134,6 @@
           <t>Res. 1154/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y30" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z30" t="inlineStr">
-        <is>
-          <t>Antes del anuncio inicial del RIGI, Josemaría ya contaba con una factibilidad de noviembre de 2020, una evaluación ambiental aprobada en abril de 2022, ingeniería, adquisición de equipos de larga entrega y USD 276 millones de gastos de capital durante 2023; Filo del Sol también poseía prefactibilidades y exploración avanzada. Estos antecedentes corresponden a los mismos depósitos y, principalmente, a la actual primera etapa basada en Josemaría. Sin embargo, la sociedad conjunta BHP–Lundin se constituyó en enero de 2025, la primera evaluación técnica unificada apareció en febrero de 2026 y la decisión final de inversión continuaba pendiente después de la aprobación.</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3500,16 +3310,6 @@
           <t>Res. 1553/2025; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y32" t="inlineStr">
-        <is>
-          <t>Ambiguo</t>
-        </is>
-      </c>
-      <c r="Z32" t="inlineStr">
-        <is>
-          <t>La norma del Proyecto Los Azules menciona que el objetivo es completar el desarrollo (factibilidad y permisos) y construir la mina y planta, lo que sugiere que hay estudios y permisos previos; sin embargo, no se identifica claramente la existencia de una operación activa previa.</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3895,16 +3695,6 @@
           <t>Res. 873/2026; Globaris; MECON</t>
         </is>
       </c>
-      <c r="Y37" t="inlineStr">
-        <is>
-          <t>Sí</t>
-        </is>
-      </c>
-      <c r="Z37" t="inlineStr">
-        <is>
-          <t>PAE ya informaba en 2024 que el esquema de GNL requería infraestructura adicional: interconexión a gasoductos troncales, estación compresora, gasoducto terrestre hasta la costa, gasoducto submarino y sistema de amarre. También indicaba que PAE y Golar habían firmado en julio de 2024 un acuerdo por 20 años para instalar el buque Hilli Episeyo en Argentina.</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4006,16 +3796,6 @@
       <c r="W38" t="inlineStr">
         <is>
           <t>Res. 1271/2025; Globaris; MECON</t>
-        </is>
-      </c>
-      <c r="Y38" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="Z38" t="inlineStr">
-        <is>
-          <t>La resolución del Proyecto Hombre Muerto Oeste (HMW) especifica una nueva producción de 12.000 t/año de carbonato de litio equivalente en la cuenca del Salar del Hombre Muerto; no se mencionan ampliaciones de proyectos previos.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
actualización 16 de agosto
</commit_message>
<xml_diff>
--- a/downloads/base_completa.xlsx
+++ b/downloads/base_completa.xlsx
@@ -355,7 +355,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:X41"/>
+  <dimension ref="A1:X42"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="16" max="16" width="20.7109375" style="2" customWidth="1"/>
@@ -4018,6 +4018,79 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Argentina LNG</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Proyecto integrado de producción y exportación de gas natural licuado: desarrollo de gas rico en Vaca Muerta, infraestructura dedicada de transporte, plantas de procesamiento y fraccionamiento y dos unidades flotantes de licuefacción (FLNG) por 12 MTPA en el Golfo San Matías.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>YPF S.A. (Argentina); Eni S.p.A. (Italia); XRG (Emiratos Árabes Unidos)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>YPF</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Petróleo y Gas</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Upstream</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Neuquén; Río Negro</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Patagonia</t>
+        </is>
+      </c>
+      <c r="L42">
+        <v>51000</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>En evaluación</t>
+        </is>
+      </c>
+      <c r="P42" s="2">
+        <v>46247</v>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>Globaris [https://app.powerbi.com/view?r=eyJrIjoiNTFjY2E4NTYtOTVlNy00YmFiLWIwYmMtNWZkMjE4OTNhYmRiIiwidCI6IjNlMDUxM2Q2LTY4ZmEtNDE2ZS04ZGUxLTZjNWNkYzMxOWZmYSIsImMiOjR9&amp;pageName=d1ee75596a51a9bde708]; YPF / Argentina LNG [https://argentina-lng.ypf.com/assets/pdf/ENG-Argentina-LNG-Adhesion-RIGI.pdf]; La Nación [https://www.lanacion.com.ar/economia/un-proyecto-por-us51000-millones-impulsado-por-ypf-solicito-la-adhesion-al-rigi-nid13082026/]; Infobae [https://www.infobae.com/economia/2026/08/13/con-una-inversion-de-usd-50000-millones-ypf-presenta-al-rigi-el-mayor-proyecto-de-su-historia-para-exportar-gas-de-vaca-muerta/]; Data Energía [https://dataenergia.ar/gas/argentina-lgn-solicitaron-la-adhesion-formal-al-rigi-para-una-inversion-historica-de-u-s-51-000-millones-202681319370]</t>
+        </is>
+      </c>
+      <c r="W42" t="inlineStr">
+        <is>
+          <t>YPF / Argentina LNG; La Nación; Infobae; Data Energía</t>
+        </is>
+      </c>
+      <c r="X42" t="inlineStr">
+        <is>
+          <t>https://argentina-lng.ypf.com/assets/pdf/ENG-Argentina-LNG-Adhesion-RIGI.pdf; https://www.lanacion.com.ar/economia/un-proyecto-por-us51000-millones-impulsado-por-ypf-solicito-la-adhesion-al-rigi-nid13082026/; https://www.infobae.com/economia/2026/08/13/con-una-inversion-de-usd-50000-millones-ypf-presenta-al-rigi-el-mayor-proyecto-de-su-historia-para-exportar-gas-de-vaca-muerta/; https://dataenergia.ar/gas/argentina-lgn-solicitaron-la-adhesion-formal-al-rigi-para-una-inversion-historica-de-u-s-51-000-millones-202681319370</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>